<commit_message>
Factibilidad: simplificar formula ROI, quitar punto de equilibrio y agregar ejemplo de costo real (guia primeros auxilios .000)
</commit_message>
<xml_diff>
--- a/public/plantilla-roi-operacion-turistica.xlsx
+++ b/public/plantilla-roi-operacion-turistica.xlsx
@@ -1,22 +1,129 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="ROI Turístico" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen general" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Guía rápida" sheetId="3" state="visible" r:id="rId3"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-09-14T19:27:24Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-14T19:27:24Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\charts\chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ingresos vs. Costos vs. Utilidad (período)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen general'!B17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumen general'!$A$18:$A$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen general'!$B$18:$B$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
@@ -270,116 +377,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Ingresos vs. Costos vs. Utilidad (período)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Resumen general'!B17</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Resumen general'!$A$18:$A$21</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Resumen general'!$B$18:$B$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>16</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -662,13 +660,30 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="ROI Turístico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen general" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Guía rápida" sheetId="3" state="visible" r:id="rId3"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -797,11 +812,16 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Guías o animadores (por persona)</t>
+          <t>Guía certificado en primeros auxilios (por persona)</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>3000</v>
+        <v>2000</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Ejemplo real: un guía certificado en primeros auxilios cuesta ~$50.000 por día; repartido en un grupo de 25 visitantes equivale a ~$2.000 por persona.</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1068,11 +1088,11 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>ROI del período</t>
+          <t>ROI del período (retorno de la inversión)</t>
         </is>
       </c>
       <c r="B43" s="10">
-        <f>IF(SUM(B28:B30)=0,0,B42/SUM(B28:B30))</f>
+        <f>IF(SUM(B28:B30)=0,0,((B36-B37-B39)-SUM(B28:B30))/SUM(B28:B30))</f>
         <v/>
       </c>
     </row>
@@ -1090,21 +1110,10 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Punto de equilibrio (visitantes)</t>
+          <t>Utilidad neta por persona</t>
         </is>
       </c>
       <c r="B45" s="9">
-        <f>IF((B9+B10)-(B13+B14+B15+B16)&gt;0,B39/((B9+B10)-(B13+B14+B15+B16)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>Utilidad neta por persona</t>
-        </is>
-      </c>
-      <c r="B46" s="9">
         <f>IF(B33&gt;0,B42/B33,0)</f>
         <v/>
       </c>
@@ -1137,7 +1146,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1253,17 +1262,6 @@
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Punto de equilibrio (visitantes)</t>
-        </is>
-      </c>
-      <c r="B14" s="9">
-        <f>'ROI Turístico'!B45</f>
-        <v/>
-      </c>
-    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -1337,7 +1335,7 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>•  Punto de equilibrio: número de visitantes mínimo para no perder dinero.</t>
+          <t>•  ROI menor a 0%: todavía no recuperas la inversión.</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>